<commit_message>
feat(audit): finalize Phase 3 discovery, Phase 4 quality audit & cross-dataset linking matrix
</commit_message>
<xml_diff>
--- a/reports/dataset_audit/dataset_audit_dashboard.xlsx
+++ b/reports/dataset_audit/dataset_audit_dashboard.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS03_Rice_Jabar" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS05_Maize_Jabar" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS06_Horticulture_SBS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linking_Feasibility_Matrix" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -603,15 +604,6 @@
           <t>Reanalysis-derived proxy, not direct in-situ ground station observation.</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -646,11 +638,6 @@
       <c r="H3" t="n">
         <v>11.73</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>PASS (METHODOLOGICAL_REFERENCE)</t>
@@ -671,13 +658,6 @@
           <t>['Aus', 'Aman', 'Boro']</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -712,11 +692,6 @@
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>PASS (REGIONAL_OUTCOME)</t>
@@ -727,8 +702,6 @@
           <t>Annual temporal grain is too coarse for daily decision advisory; requires linkage with daily weather.</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="n">
         <v>27</v>
       </c>
@@ -737,11 +710,6 @@
           <t>KUINTAL PER HEKTAR</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -776,11 +744,6 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>PASS (AGROCLIMATE_BENCHMARK)</t>
@@ -791,19 +754,12 @@
           <t>Derived from ERA5-Seamless; 0.5° spatial grid is coarser than native 0.1° AgERA5.</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>612</v>
       </c>
       <c r="U5" t="n">
         <v>12</v>
       </c>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -838,11 +794,6 @@
       <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>PASS (REGIONAL_OUTCOME)</t>
@@ -853,8 +804,6 @@
           <t>Official published series is at regency level (Kab. Subang included); subdistrict (kecamatan) breakdown had server-side 502 error on government API.</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="n">
         <v>27</v>
       </c>
@@ -863,13 +812,9 @@
           <t>KUINTAL/HEKTAR</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
         <v>8</v>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -904,11 +849,6 @@
       <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>PASS (HORTICULTURE_OUTCOME)</t>
@@ -919,17 +859,11 @@
           <t>Aggregated productivity dataset; does NOT contain disease incidence/severity labels.</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>KUINTAL PER HEKTAR</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
         <v>55</v>
       </c>
@@ -4040,7 +3974,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>24 agricultural variables, daily time-series, native 0.1 deg grid</t>
@@ -4126,7 +4059,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>24 agricultural variables, daily time-series, native 0.1 deg grid</t>
@@ -4212,7 +4144,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>Full replication archive with yield and climate panel for 64 districts</t>
@@ -4298,7 +4229,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>Full replication archive with yield and climate panel for 64 districts</t>
@@ -4384,7 +4314,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>Full replication archive with yield and climate panel for 64 districts</t>
@@ -4470,7 +4399,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>Full replication archive with yield and climate panel for 64 districts</t>
@@ -4556,7 +4484,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>Padi Total (Sawah + Ladang)</t>
@@ -4642,7 +4569,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>Raw API Response</t>
@@ -4728,7 +4654,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>Padi Sawah (Wetland Rice)</t>
@@ -4814,7 +4739,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>Padi Ladang (Dryland Rice)</t>
@@ -4900,7 +4824,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>Combined indicators 2016-2025 (60 MB)</t>
@@ -4986,7 +4909,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>Quality-controlled weather 2016-2025 (15.5 MB)</t>
@@ -5072,7 +4994,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>612 Indonesian terrestrial grid coordinates</t>
@@ -5158,7 +5079,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
           <t>12 derived agroclimatic indicator definitions</t>
@@ -5244,7 +5164,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>Produktivitas jagung 2015-2022 across 27 kab/kota incl Subang</t>
@@ -5330,7 +5249,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>Raw API Response</t>
@@ -5416,7 +5334,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>Produktivitas Sayuran &amp; Buah Semusim 2017-2025</t>
@@ -5502,7 +5419,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>Raw API Response SBS</t>
@@ -5588,7 +5504,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>Produksi Sayuran per Komoditas Kab/Kota 2013-2024</t>
@@ -5674,7 +5589,6 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>Raw API Response Produksi</t>
@@ -24613,4 +24527,470 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>linking_pair_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>target_engine</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>weather_source</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>outcome_source</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>weather_period</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>outcome_period</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>overlap_temporal_years</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>overlap_period</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>weather_spatial_grain</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>outcome_spatial_grain</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>overlap_spatial_status</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>grain_gap</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>linking_feasibility_rating</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>feature_engineering_strategy</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>key_risk_factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>LINK_01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rice Decision Engine (Padi)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DS03 (Produktivitas Padi Jabar Distanhor)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2015-01-01 s.d. 2024-12-31</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2015 s.d. 2020</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2015–2020</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) 7 Sentra Jabar</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>27 Kabupaten/Kota Se-Jawa Barat</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>MATCHED (7 Kabupaten Utama Beririsan Sempurna)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Yield</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Agregasi cuaca harian ke siklus tanam 120 hari (Musim Hujan MH &amp; Musim Kemarau MK) untuk 27 sentra pangan.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Waterlogging/banjir fase seedling dan heat stress fase flowering/reproduktif.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LINK_02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Maize Decision Engine (Jagung)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DS05 (Produktivitas Jagung Jabar &amp; Subang)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2015-01-01 s.d. 2024-12-31</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2015 s.d. 2022</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2015–2022</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) Purwakarta/Bekasi/Karawang buffer</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Kabupaten Subang &amp; 27 Kab/Kota</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>MATCHED (Kabupaten Subang Terisolasi 8 Tahun Penuh)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Yield</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Akumulasi GDD (Growing Degree Days) &amp; Defisit Air (WSI/VPD) pada jendela 90–110 hari fase vegetatif hingga pembentukan biji.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Drought stress (CDD tinggi) dan kelembaban ekstrem saat pengisian biji.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LINK_03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Horticulture Decision Engine (Cabai)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DS06 (Produktivitas SBS Cabai Rawit &amp; Besar)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2015-01-01 s.d. 2024-12-31</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2017 s.d. 2024</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2017–2024</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) Sentra Hortikultura (Bandung/Sukabumi/Tasikmalaya)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Jawa Barat (Cabai Rawit &amp; Cabai Besar)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>MATCHED (Provinsi &amp; Sentra Dataran Tinggi/Sedang)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Yield</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>MODERATE_TO_HIGH</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Model Yield: Agregasi cuaca harian multi-petik. Model Penyakit (OPT): Rule-based mechanistic weather threshold (RH &gt; 90% + suhu 24-28°C durasi 3 hari).</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Penyakit antraknosa (patek) dan busuk buah saat periode basah berkepanjangan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LINK_04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Extreme Climate Early Warning Layer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DS04 (Indonesia Nationwide Agroclimatic)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2016 s.d. 2025</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2015-01-01 s.d. 2024-12-31</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2016–2024</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Grid 0,5° (~55 km) 14 Titik Jawa Barat</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) 7 Titik Sentra Jawa Barat</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>MATCHED (Cross-grid Validation Jawa Barat)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Daily Indicators vs Daily AgERA5</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>VERY_HIGH</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Validasi silang ambang batas hari kering berurutan (CDD), hari basah (CWD), dan evapotranspirasi FAO-56 untuk kalibrasi alert dini.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Anomali iklim ekstrem makro (El Niño / La Niña / IOD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LINK_05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Methodological &amp; Panel Benchmark</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DS02 Weather Covariates (BRRI Bangladesh)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DS02 Audited Rice Yield (BRRI Bangladesh)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2015–2024 (Season-level climate)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2015-16 s.d. 2023-24 (3 Musim Tanam)</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2015–2024</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>64 Distrik Administratif Bangladesh</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>64 Distrik Administratif Bangladesh</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>MATCHED (Panel Seimbang 1.728 Baris)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Seasonal Climate vs Seasonal District Yield</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>VERY_HIGH</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Regresi panel Fixed Effects (FE) &amp; Random Effects (RE) sebagai tolok ukur spesifikasi model sebelum diterapkan ke data Jabar.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Efek musim tanam asimetris (Boro irigasi vs Aman monsun).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(audit): complete phase 5 empirical verification, fix maize trend bug, and clean repo structure
- Fix Subang maize R2 bug from 1.000 to 0.739 and compute 27 regency trends
- Audit 15 research papers and separate temperate vs local evidence
- Acquire official soybean data and select Tomato for 4-crop portfolio
- Extract true ADM2 polygon centroids and audit AgERA5 cell counts
- Specify decision engine JSON output schema in docs/engine_output_schema.md
- Consolidate figures into reports/figures/ and clean up obsolete scratch files
</commit_message>
<xml_diff>
--- a/reports/dataset_audit/dataset_audit_dashboard.xlsx
+++ b/reports/dataset_audit/dataset_audit_dashboard.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:Y7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,55 +492,60 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>effective_n_matched</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>disposition</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>limitations</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>panel_keys</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>seasons</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>regions_count</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>grid_points_count</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>derived_indicators_count</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>subang_records_count</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>commodities_count</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>chili_commodities</t>
         </is>
@@ -554,7 +559,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AgERA5 Time-Series (Primary Weather Backbone)</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -596,14 +601,28 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>N_eff = 42 (Padi), 56 (Jagung)</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Reanalysis-derived proxy, not direct in-situ ground station observation.</t>
-        </is>
-      </c>
+          <t>PASS (PRIMARY_WEATHER_BACKBONE)</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Data reanalisis grid spasial 0,1° (~10 km); saat ini 7 titik di Jabar. Subang belum terhubung langsung.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -638,26 +657,43 @@
       <c r="H3" t="n">
         <v>11.73</v>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>PASS (METHODOLOGICAL_REFERENCE)</t>
+          <t>N = 1.728 baris panel seimbang (64 distrik x 3 musim x 9 thn)</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Geographically non-local; represents Bangladesh agricultural systems, not direct validation for West Java.</t>
+          <t>PASS (METHODOLOGICAL_BENCHMARK)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>Data internasional Bangladesh; tolok ukur ekonometrika regresi panel iklim vs yield, bukan kalibrasi lokal Jabar.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>district x crop x crop_year</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>['Aus', 'Aman', 'Boro']</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -692,24 +728,41 @@
       <c r="H4" t="n">
         <v>0</v>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>PASS (REGIONAL_OUTCOME)</t>
+          <t>N_eff = 42 baris (7 kab beririsan dg AgERA5; expandable ke 162)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Annual temporal grain is too coarse for daily decision advisory; requires linkage with daily weather.</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
+          <t>PASS (REGIONAL_RICE_OUTCOME)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Data luaran tahunan murni tanpa pemisahan musim MH/MK. Memerlukan agregasi kalender tahunan atau 2 musim kumulatif.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="n">
         <v>27</v>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>KUINTAL PER HEKTAR</t>
-        </is>
-      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>KUINTAL PER HEKTAR</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -744,22 +797,39 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
+          <t>612 titik terestrial Indonesia (14 titik Jawa Barat)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>PASS (AGROCLIMATE_BENCHMARK)</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Derived from ERA5-Seamless; 0.5° spatial grid is coarser than native 0.1° AgERA5.</t>
-        </is>
-      </c>
-      <c r="T5" t="n">
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Turunan reanalisis ERA5-Seamless (0,5° grid); membuktikan konsistensi ECMWF (r=0,85), bukan validasi ground-truth BMKG.</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
         <v>612</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>12</v>
       </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -794,27 +864,43 @@
       <c r="H6" t="n">
         <v>0</v>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>PASS (REGIONAL_OUTCOME)</t>
+          <t>N_eff = 0 (Subang Unmatched pada 7 titik AgERA5 saat ini; 56 untuk 7 kab lain)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Official published series is at regency level (Kab. Subang included); subdistrict (kecamatan) breakdown had server-side 502 error on government API.</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
+          <t>PASS (REGIONAL_MAIZE_OUTCOME)</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Patahan struktural 2020-2022 (+56,4% dlm 2 thn) memerlukan detrending linear (+4,93 ku/ha/thn); variasi cuaca pada residu CV 11,42%.</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="n">
         <v>27</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>KUINTAL/HEKTAR</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
         <v>8</v>
       </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -849,27 +935,43 @@
       <c r="H7" t="n">
         <v>0</v>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>PASS (HORTICULTURE_OUTCOME)</t>
+          <t>N_eff = 8 baris per varian (Agregat Provinsi Jawa Barat)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Aggregated productivity dataset; does NOT contain disease incidence/severity labels.</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>KUINTAL PER HEKTAR</t>
-        </is>
-      </c>
-      <c r="W7" t="n">
+          <t>PASS (REGIONAL_HORTICULTURE_OUTCOME)</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Data luaran agregat provinsi (N=8); label penyakit/OPT absen. Dilarang melatih ML penyakit; wajib gunakan IFWC berbasis proksi T - Td.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>KUINTAL PER HEKTAR</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="n">
         <v>55</v>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>['CABAI BESAR', 'CABAI RAWIT', 'CABAI KERITING', 'Cabai Besar (Group)', 'Cabai Besar/ TW / Teropong', 'Cabai Keriting', 'Cabai Rawit']</t>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>['CABAI BESAR', 'CABAI RAWIT']</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3961,7 +4063,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:16.915217</t>
+          <t>2026-10-10T10:14:43.780037</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3974,9 +4076,10 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>24 agricultural variables, daily time-series, native 0.1 deg grid</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (PILOT_BANDUNG_ALL_VARS_2023.CSV)</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4149,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:16.919937</t>
+          <t>2026-10-10T10:14:43.831644</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -4059,84 +4162,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>24 agricultural variables, daily time-series, native 0.1 deg grid</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (BANDUNG)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DS02</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Methodological/Comparison Benchmark</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>10.17632/h94z4ftts2.1</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>data/raw/DS02_bangladesh_rice_panel/Growing_Season_Climate_Rice_Bangladesh_Mendeley_Replication_v1.zip</t>
+          <t>data/raw/DS01_agera5\agera5_karawang_2015_2024.csv</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Growing_Season_Climate_Rice_Bangladesh_Mendeley_Replication_v1.zip</t>
+          <t>agera5_karawang_2015_2024.csv</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ZIP</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>10029466</v>
+        <v>1000702</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>8abd695a609060d44271d7473a87fc71c5c6c50c833e618ce35a5c0444801d6f</t>
+          <t>aa6b777e61dbd4c4ffd716b6de8c2431cb208b55105734e14a08962adcc4d41c</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:16.949643</t>
+          <t>2026-10-10T10:14:43.871774</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -4144,84 +4248,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Full replication archive with yield and climate panel for 64 districts</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (KARAWANG)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DS02</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Methodological/Comparison Benchmark</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>10.17632/h94z4ftts2.1</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>data/raw/DS02_bangladesh_rice_panel/README.txt</t>
+          <t>data/raw/DS01_agera5\agera5_tasikmalaya_2015_2024.csv</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>README.txt</t>
+          <t>agera5_tasikmalaya_2015_2024.csv</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>TXT</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>3569</v>
+        <v>993146</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>7688c71da184c3588feaf1052604e76a54c47a765d0a5d24de26f9a52b006d9a</t>
+          <t>09c1aa61eeb56ce2773bdfb9d8860e089633d1ac2a7508c58ff5c0468ad83ace</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:16.952167</t>
+          <t>2026-10-10T10:14:43.898971</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -4229,61 +4334,62 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Full replication archive with yield and climate panel for 64 districts</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (TASIKMALAYA)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DS02</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Methodological/Comparison Benchmark</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10.17632/h94z4ftts2.1</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>data/raw/DS02_bangladesh_rice_panel/extracted/Growing_Season_Climate_Rice_Bangladesh_Replication/Rice_Yield_2015_2024_Audited.csv</t>
+          <t>data/raw/DS01_agera5\agera5_sukabumi_2015_2024.csv</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Rice_Yield_2015_2024_Audited.csv</t>
+          <t>agera5_sukabumi_2015_2024.csv</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -4292,21 +4398,21 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>804697</v>
+        <v>995878</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>5103ab5e480cbd34842e55761f3aa7d4cea179ff32616360d2910906e90ffbce</t>
+          <t>174c101ceee54e82121b4f43269a1da5615867e81a139b55b6864e0935a09fe8</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:16.990810</t>
+          <t>2026-10-10T10:14:43.926937</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -4314,61 +4420,62 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Full replication archive with yield and climate panel for 64 districts</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (SUKABUMI)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DS02</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Methodological/Comparison Benchmark</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>10.17632/h94z4ftts2.1</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>data/raw/DS02_bangladesh_rice_panel/extracted/Growing_Season_Climate_Rice_Bangladesh_Replication/03_merge/Phase5_Final_Merged_Primary_2015_2024.csv</t>
+          <t>data/raw/DS01_agera5\agera5_cirebon_2015_2024.csv</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Phase5_Final_Merged_Primary_2015_2024.csv</t>
+          <t>agera5_cirebon_2015_2024.csv</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -4377,21 +4484,21 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>1360631</v>
+        <v>999859</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>4ab44b9a2236327e6a224cc181c2b15a8cf25be59257b73e18b90b85c98dd6cd</t>
+          <t>43edea748d0fc3d0491debd668a85a49989f93c314e89d5a8b4c09a5f4ebeae6</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.016595</t>
+          <t>2026-10-10T10:14:43.948291</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -4399,61 +4506,62 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Full replication archive with yield and climate panel for 64 districts</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (CIREBON)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DS03</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>West Java Rice Productivity by Regency/City</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Regional Rice Outcome Target</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>OD-18103 (2015-2020)</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_jabar.csv</t>
+          <t>data/raw/DS01_agera5\agera5_purwakarta_2015_2024.csv</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>produktivitas_padi_jabar.csv</t>
+          <t>agera5_purwakarta_2015_2024.csv</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -4462,21 +4570,21 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>11479</v>
+        <v>1006801</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>c03b11b683b131d8ba8c7b7d8e065fbc5707bc2fe28e243cb72a4a4f7343f0bd</t>
+          <t>5c098d7ade5e40090591367cb5e79e8bdd3b6ed1e9903710234fec50f78c9b63</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.037426</t>
+          <t>2026-10-10T10:14:43.969098</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -4484,84 +4592,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Padi Total (Sawah + Ladang)</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (PURWAKARTA)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DS03</t>
+          <t>DS01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>West Java Rice Productivity by Regency/City</t>
+          <t>AgERA5 Agrometeorological Indicators Time-Series</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Regional Rice Outcome Target</t>
+          <t>Primary Weather Backbone</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
+          <t>https://cds.climate.copernicus.eu/datasets/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://cds.climate.copernicus.eu/api/retrieve/v1/processes/sis-agrometeorological-indicators-timeseries</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Copernicus Climate Change Service (ECMWF)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>OD-18103 (2015-2020)</t>
+          <t>AgERA5 v2.0</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>Copernicus Open Access</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_jabar.json</t>
+          <t>data/raw/DS01_agera5\agera5_bekasi_2015_2024.csv</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>produktivitas_padi_jabar.json</t>
+          <t>agera5_bekasi_2015_2024.csv</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L9" t="n">
-        <v>33433</v>
+        <v>1004572</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>5063402756006a750ac2639f82c21254e8468bbf6e5926750580fc7116b477eb</t>
+          <t>8cfeeb7516e1f15cca93f319f364fe57df760ee2fed6c4fd657d8883e8440e65</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.039423</t>
+          <t>2026-10-10T10:14:43.994591</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>API_AUTOMATED</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4569,84 +4678,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Raw API Response</t>
+          <t>24 agricultural variables, daily 2015-2024, native 0.1 deg grid (BEKASI)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DS03</t>
+          <t>DS02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>West Java Rice Productivity by Regency/City</t>
+          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Regional Rice Outcome Target</t>
+          <t>Methodological/Comparison Benchmark</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
+          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Mendeley Data / Elsevier</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>OD-18103 (2015-2020)</t>
+          <t>10.17632/h94z4ftts2.1</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_sawah_jabar.csv</t>
+          <t>data/raw/DS02_bangladesh_rice_panel/Growing_Season_Climate_Rice_Bangladesh_Mendeley_Replication_v1.zip</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>produktivitas_padi_sawah_jabar.csv</t>
+          <t>Growing_Season_Climate_Rice_Bangladesh_Mendeley_Replication_v1.zip</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>ZIP</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>11479</v>
+        <v>10029466</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>fb64da4d527fc1eabaab16bfc21bd4fcfde16040a523c73a5599a50b74cf6ec8</t>
+          <t>8abd695a609060d44271d7473a87fc71c5c6c50c833e618ce35a5c0444801d6f</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.065077</t>
+          <t>2026-10-10T10:14:44.024227</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>HTTP_API_DIRECT</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4654,84 +4764,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Padi Sawah (Wetland Rice)</t>
+          <t>Full replication archive with yield and climate panel for 64 districts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DS03</t>
+          <t>DS02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>West Java Rice Productivity by Regency/City</t>
+          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Regional Rice Outcome Target</t>
+          <t>Methodological/Comparison Benchmark</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
+          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Mendeley Data / Elsevier</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>OD-18103 (2015-2020)</t>
+          <t>10.17632/h94z4ftts2.1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_ladang_jabar.csv</t>
+          <t>data/raw/DS02_bangladesh_rice_panel/README.txt</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>produktivitas_padi_ladang_jabar.csv</t>
+          <t>README.txt</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>TXT</t>
         </is>
       </c>
       <c r="L11" t="n">
-        <v>11382</v>
+        <v>3569</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>c24cbb8073d2879d79180ddc099c4f82a7632b04d60049ad105e0ed04abe4f02</t>
+          <t>7688c71da184c3588feaf1052604e76a54c47a765d0a5d24de26f9a52b006d9a</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.105921</t>
+          <t>2026-10-10T10:14:44.027777</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>HTTP_API_DIRECT</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4739,36 +4850,37 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Padi Ladang (Dryland Rice)</t>
+          <t>Full replication archive with yield and climate panel for 64 districts</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DS04</t>
+          <t>DS02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Indonesia Nationwide Agroclimatic Dataset</t>
+          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Agroclimate Reference &amp; Comparison Backbone</t>
+          <t>Methodological/Comparison Benchmark</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
+          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
+          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -4778,7 +4890,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10.17632/3pfbdbzfff.1</t>
+          <t>10.17632/h94z4ftts2.1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4788,30 +4900,30 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>data/raw/DS04_indonesia_agroclimatic/agroclimate_with_indicators.parquet</t>
+          <t>data/raw/DS02_bangladesh_rice_panel/extracted/Growing_Season_Climate_Rice_Bangladesh_Replication/Rice_Yield_2015_2024_Audited.csv</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>agroclimate_with_indicators.parquet</t>
+          <t>Rice_Yield_2015_2024_Audited.csv</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>PARQUET</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>60007977</v>
+        <v>804697</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>3c6475a4b6fb11a138038fb216cb59c784bccdb6bb38a8f4c0456c39d41984cc</t>
+          <t>5103ab5e480cbd34842e55761f3aa7d4cea179ff32616360d2910906e90ffbce</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.278350</t>
+          <t>2026-10-10T10:14:44.031776</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -4824,36 +4936,37 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Combined indicators 2016-2025 (60 MB)</t>
+          <t>Full replication archive with yield and climate panel for 64 districts</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DS04</t>
+          <t>DS02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indonesia Nationwide Agroclimatic Dataset</t>
+          <t>Bangladesh Rice Climate–Yield Panel Replication Archive</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Agroclimate Reference &amp; Comparison Backbone</t>
+          <t>Methodological/Comparison Benchmark</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
+          <t>https://data.mendeley.com/datasets/h94z4ftts2/1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
+          <t>https://data.mendeley.com/public-files/datasets/h94z4ftts2/files/1aa46123-9324-4adf-9f4a-756cf2bfefb6/file_downloaded</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -4863,7 +4976,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10.17632/3pfbdbzfff.1</t>
+          <t>10.17632/h94z4ftts2.1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4873,30 +4986,30 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>data/raw/DS04_indonesia_agroclimatic/agroclimate_qc.parquet</t>
+          <t>data/raw/DS02_bangladesh_rice_panel/extracted/Growing_Season_Climate_Rice_Bangladesh_Replication/03_merge/Phase5_Final_Merged_Primary_2015_2024.csv</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>agroclimate_qc.parquet</t>
+          <t>Phase5_Final_Merged_Primary_2015_2024.csv</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>PARQUET</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>15531963</v>
+        <v>1360631</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>ffda66c3ff070cde73f456fbc02d9577a27e960cbba69e222a57db629c897a66</t>
+          <t>4ab44b9a2236327e6a224cc181c2b15a8cf25be59257b73e18b90b85c98dd6cd</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.318828</t>
+          <t>2026-10-10T10:14:44.038643</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -4909,61 +5022,62 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Quality-controlled weather 2016-2025 (15.5 MB)</t>
+          <t>Full replication archive with yield and climate panel for 64 districts</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DS04</t>
+          <t>DS03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Indonesia Nationwide Agroclimatic Dataset</t>
+          <t>West Java Rice Productivity by Regency/City</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Agroclimate Reference &amp; Comparison Backbone</t>
+          <t>Regional Rice Outcome Target</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
+          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10.17632/3pfbdbzfff.1</t>
+          <t>OD-18103 (2015-2020)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Government Open Data</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>data/raw/DS04_indonesia_agroclimatic/grid_points.csv</t>
+          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_jabar.csv</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>grid_points.csv</t>
+          <t>produktivitas_padi_jabar.csv</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -4972,21 +5086,21 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>18783</v>
+        <v>11479</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>746130ecf92dfcfec73fd2d3ae3096bd3a1635d395b7700544021cc1f6ed4b3d</t>
+          <t>c03b11b683b131d8ba8c7b7d8e065fbc5707bc2fe28e243cb72a4a4f7343f0bd</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.320853</t>
+          <t>2026-10-10T10:14:44.038643</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>SESSION_REST_API</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -4994,84 +5108,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>612 Indonesian terrestrial grid coordinates</t>
+          <t>Padi Total (Sawah + Ladang)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DS04</t>
+          <t>DS03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Indonesia Nationwide Agroclimatic Dataset</t>
+          <t>West Java Rice Productivity by Regency/City</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Agroclimate Reference &amp; Comparison Backbone</t>
+          <t>Regional Rice Outcome Target</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
+          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Mendeley Data / Elsevier</t>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10.17632/3pfbdbzfff.1</t>
+          <t>OD-18103 (2015-2020)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CC BY 4.0</t>
+          <t>Government Open Data</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>data/raw/DS04_indonesia_agroclimatic/indicator_definitions.csv</t>
+          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_jabar.json</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>indicator_definitions.csv</t>
+          <t>produktivitas_padi_jabar.json</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>1268</v>
+        <v>33433</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>28fc356fd418d6f4c0ace4814a3f6a669fbf678f390e046288550112e7ea0aff</t>
+          <t>5063402756006a750ac2639f82c21254e8468bbf6e5926750580fc7116b477eb</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.322292</t>
+          <t>2026-10-10T10:14:44.043041</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>HTTP_API_DIRECT</t>
+          <t>SESSION_REST_API</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -5079,36 +5194,37 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>12 derived agroclimatic indicator definitions</t>
+          <t>Raw API Response</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DS05</t>
+          <t>DS03</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Subang &amp; West Java Maize Productivity</t>
+          <t>West Java Rice Productivity by Regency/City</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Regional Maize Outcome Target</t>
+          <t>Regional Rice Outcome Target</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-jagung-menurut-kecamatan-di-kabupaten-subang</t>
+          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-jagung-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -5118,7 +5234,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Distanhor Jabar (2015-2022)</t>
+          <t>OD-18103 (2015-2020)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -5128,12 +5244,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>data/raw/DS05_subang_maize_productivity/produktivitas_jagung_jabar.csv</t>
+          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_sawah_jabar.csv</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>produktivitas_jagung_jabar.csv</t>
+          <t>produktivitas_padi_sawah_jabar.csv</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -5142,16 +5258,16 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>14349</v>
+        <v>11479</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>45e19886627ee04582ef997b289594cecc222d90be2eeee9f55a049244beaf3d</t>
+          <t>fb64da4d527fc1eabaab16bfc21bd4fcfde16040a523c73a5599a50b74cf6ec8</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.353085</t>
+          <t>2026-10-10T10:14:44.044587</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -5164,36 +5280,37 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Produktivitas jagung 2015-2022 across 27 kab/kota incl Subang</t>
+          <t>Padi Sawah (Wetland Rice)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DS05</t>
+          <t>DS03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Subang &amp; West Java Maize Productivity</t>
+          <t>West Java Rice Productivity by Regency/City</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Regional Maize Outcome Target</t>
+          <t>Regional Rice Outcome Target</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://data.go.id/dataset/dataset/produktivitas-jagung-menurut-kecamatan-di-kabupaten-subang</t>
+          <t>https://data.go.id/dataset/dataset/produktivitas-padi-berdasarkan-kabupaten-kota-di-jawa-barat</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-jagung-berdasarkan-kabupatenkota-di-jawa-barat</t>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-padi-berdasarkan-kabupatenkota-di-jawa-barat</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -5203,7 +5320,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Distanhor Jabar (2015-2022)</t>
+          <t>OD-18103 (2015-2020)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -5213,30 +5330,30 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>data/raw/DS05_subang_maize_productivity/produktivitas_jagung_jabar.json</t>
+          <t>data/raw/DS03_west_java_rice_productivity/produktivitas_padi_ladang_jabar.csv</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>produktivitas_jagung_jabar.json</t>
+          <t>produktivitas_padi_ladang_jabar.csv</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>CSV</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>43388</v>
+        <v>11382</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2b9286ae16e2eae9418761436104f5a675b444c85452cf189e10df287d2684c5</t>
+          <t>c24cbb8073d2879d79180ddc099c4f82a7632b04d60049ad105e0ed04abe4f02</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.355771</t>
+          <t>2026-10-10T10:14:44.046076</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -5249,84 +5366,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Raw API Response</t>
+          <t>Padi Ladang (Dryland Rice)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DS06</t>
+          <t>DS04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+          <t>Indonesia Nationwide Agroclimatic Dataset</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Regional Horticulture Outcome Target</t>
+          <t>Agroclimate Reference &amp; Comparison Backbone</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Mendeley Data / Elsevier</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Distanhor Jabar SBS (2017-2025)</t>
+          <t>10.17632/3pfbdbzfff.1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>data/raw/DS06_west_java_horticulture/produktivitas_sbs_jabar.csv</t>
+          <t>data/raw/DS04_indonesia_agroclimatic/agroclimate_with_indicators.parquet</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>produktivitas_sbs_jabar.csv</t>
+          <t>agroclimate_with_indicators.parquet</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>CSV</t>
+          <t>PARQUET</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>13511</v>
+        <v>60007977</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>dbe2065e55fbd1003eafdd5add3588b1459a4018370aed19093c8c29ca2c5512</t>
+          <t>3c6475a4b6fb11a138038fb216cb59c784bccdb6bb38a8f4c0456c39d41984cc</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.369376</t>
+          <t>2026-10-10T10:14:44.200888</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>HTTP_API_DIRECT</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -5334,84 +5452,85 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Produktivitas Sayuran &amp; Buah Semusim 2017-2025</t>
+          <t>Combined indicators 2016-2025 (60 MB)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DS06</t>
+          <t>DS04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+          <t>Indonesia Nationwide Agroclimatic Dataset</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Regional Horticulture Outcome Target</t>
+          <t>Agroclimate Reference &amp; Comparison Backbone</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Mendeley Data / Elsevier</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Distanhor Jabar SBS (2017-2025)</t>
+          <t>10.17632/3pfbdbzfff.1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>data/raw/DS06_west_java_horticulture/produktivitas_sbs_jabar.json</t>
+          <t>data/raw/DS04_indonesia_agroclimatic/agroclimate_qc.parquet</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>produktivitas_sbs_jabar.json</t>
+          <t>agroclimate_qc.parquet</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PARQUET</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>36979</v>
+        <v>15531963</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>760810a2ece8f77dd1cd16b71fd919b2c4b7422b41abadb7dd8620d83c4cfae5</t>
+          <t>ffda66c3ff070cde73f456fbc02d9577a27e960cbba69e222a57db629c897a66</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.371894</t>
+          <t>2026-10-10T10:14:44.278367</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>HTTP_API_DIRECT</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5419,61 +5538,62 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Raw API Response SBS</t>
+          <t>Quality-controlled weather 2016-2025 (15.5 MB)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DS06</t>
+          <t>DS04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+          <t>Indonesia Nationwide Agroclimatic Dataset</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Regional Horticulture Outcome Target</t>
+          <t>Agroclimate Reference &amp; Comparison Backbone</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+          <t>Mendeley Data / Elsevier</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Distanhor Jabar SBS (2017-2025)</t>
+          <t>10.17632/3pfbdbzfff.1</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Government Open Data</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>data/raw/DS06_west_java_horticulture/produksi_sayuran_komoditas_jabar.csv</t>
+          <t>data/raw/DS04_indonesia_agroclimatic/grid_points.csv</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>produksi_sayuran_komoditas_jabar.csv</t>
+          <t>grid_points.csv</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -5482,21 +5602,21 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>63215</v>
+        <v>18783</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>646f8ed128216ee388425311468ffea8623c2be8504bba2526c74d367df5b7b2</t>
+          <t>746130ecf92dfcfec73fd2d3ae3096bd3a1635d395b7700544021cc1f6ed4b3d</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-10-10T10:08:17.387635</t>
+          <t>2026-10-10T10:14:44.279366</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>SESSION_REST_API</t>
+          <t>HTTP_API_DIRECT</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -5504,92 +5624,610 @@
           <t>DOWNLOADED</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Produksi Sayuran per Komoditas Kab/Kota 2013-2024</t>
+          <t>612 Indonesian terrestrial grid coordinates</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>DS04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Indonesia Nationwide Agroclimatic Dataset</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Agroclimate Reference &amp; Comparison Backbone</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://data.mendeley.com/datasets/3pfbdbzfff/1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://data.mendeley.com/public-files/datasets/3pfbdbzfff/files/.../file_downloaded</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Mendeley Data / Elsevier</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>10.17632/3pfbdbzfff.1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>data/raw/DS04_indonesia_agroclimatic/indicator_definitions.csv</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>indicator_definitions.csv</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>1268</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>28fc356fd418d6f4c0ace4814a3f6a669fbf678f390e046288550112e7ea0aff</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.280372</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>HTTP_API_DIRECT</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>12 derived agroclimatic indicator definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DS05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Subang &amp; West Java Maize Productivity</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Regional Maize Outcome Target</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://data.go.id/dataset/dataset/produktivitas-jagung-menurut-kecamatan-di-kabupaten-subang</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-jagung-berdasarkan-kabupatenkota-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Distanhor Jabar (2015-2022)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Government Open Data</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>data/raw/DS05_subang_maize_productivity/produktivitas_jagung_jabar.csv</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>produktivitas_jagung_jabar.csv</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>14349</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>45e19886627ee04582ef997b289594cecc222d90be2eeee9f55a049244beaf3d</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.282382</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>SESSION_REST_API</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Produktivitas jagung 2015-2022 across 27 kab/kota incl Subang</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DS05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Subang &amp; West Java Maize Productivity</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Regional Maize Outcome Target</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://data.go.id/dataset/dataset/produktivitas-jagung-menurut-kecamatan-di-kabupaten-subang</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-jagung-berdasarkan-kabupatenkota-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Distanhor Jabar (2015-2022)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Government Open Data</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>data/raw/DS05_subang_maize_productivity/produktivitas_jagung_jabar.json</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>produktivitas_jagung_jabar.json</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>43388</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2b9286ae16e2eae9418761436104f5a675b444c85452cf189e10df287d2684c5</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.285914</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>SESSION_REST_API</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Raw API Response</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>DS06</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Regional Horticulture Outcome Target</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Distanhor Jabar SBS (2017-2025)</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Government Open Data</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>data/raw/DS06_west_java_horticulture/produktivitas_sbs_jabar.csv</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>produktivitas_sbs_jabar.csv</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>13511</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>dbe2065e55fbd1003eafdd5add3588b1459a4018370aed19093c8c29ca2c5512</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.286911</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>SESSION_REST_API</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Produktivitas Sayuran &amp; Buah Semusim 2017-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DS06</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Regional Horticulture Outcome Target</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Distanhor Jabar SBS (2017-2025)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Government Open Data</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>data/raw/DS06_west_java_horticulture/produktivitas_sbs_jabar.json</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>produktivitas_sbs_jabar.json</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>36979</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>760810a2ece8f77dd1cd16b71fd919b2c4b7422b41abadb7dd8620d83c4cfae5</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.287910</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>SESSION_REST_API</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Raw API Response SBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DS06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Regional Horticulture Outcome Target</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Distanhor Jabar SBS (2017-2025)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Government Open Data</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>data/raw/DS06_west_java_horticulture/produksi_sayuran_komoditas_jabar.csv</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>produksi_sayuran_komoditas_jabar.csv</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>63215</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>646f8ed128216ee388425311468ffea8623c2be8504bba2526c74d367df5b7b2</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.288916</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>SESSION_REST_API</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>DOWNLOADED</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Produksi Sayuran per Komoditas Kab/Kota 2013-2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DS06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>West Java Seasonal Vegetables &amp; Fruit (SBS) Productivity</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Regional Horticulture Outcome Target</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://opendata.jabarprov.go.id/id/dataset/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://galura.jabarprov.go.id/api/bigdata/produktivitas-sayuran-dan-buah-buahan-semusim-sbs-berdasarkan-komoditi-di-jawa-barat</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Dinas Tanaman Pangan dan Hortikultura Jawa Barat</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Distanhor Jabar SBS (2017-2025)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Government Open Data</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>data/raw/DS06_west_java_horticulture/produksi_sayuran_komoditas_jabar.json</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>produksi_sayuran_komoditas_jabar.json</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>JSON</t>
         </is>
       </c>
-      <c r="L21" t="n">
+      <c r="L27" t="n">
         <v>208471</v>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>9abf68e0bb141c97e57edf48b4d4651aa0d5e17c913343a27fa36429863c09b1</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>2026-10-10T10:08:17.389558</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-10-10T10:14:44.292960</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>SESSION_REST_API</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>DOWNLOADED</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
         <is>
           <t>Raw API Response Produksi</t>
         </is>
@@ -24535,7 +25173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24551,67 +25189,52 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>evidence_tier</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>weather_source</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>outcome_source</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>weather_period</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>outcome_period</t>
+          <t>temporal_overlap</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>overlap_temporal_years</t>
+          <t>spatial_overlap_status</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>overlap_period</t>
+          <t>effective_n_matched</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>weather_spatial_grain</t>
+          <t>effective_n_strict_kabupaten</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>outcome_spatial_grain</t>
+          <t>expected_signal_literature</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>overlap_spatial_status</t>
+          <t>linking_feasibility</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>grain_gap</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>linking_feasibility_rating</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>feature_engineering_strategy</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>key_risk_factor</t>
+          <t>grain_gap_mitigation</t>
         </is>
       </c>
     </row>
@@ -24623,70 +25246,53 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rice Decision Engine (Padi)</t>
+          <t>Rice (Padi)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+          <t>TIER_A (Data-Learned Regression)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DS03 (Produktivitas Padi Jabar Distanhor)</t>
+          <t>AgERA5 (DS01)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2015-01-01 s.d. 2024-12-31</t>
+          <t>Distanhor Padi Jabar (DS03)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2015 s.d. 2020</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2015–2020</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Grid 0,1° (~10 km) 7 Sentra Jabar</t>
-        </is>
+          <t>2015–2020 (6 Tahun)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PARTIAL (7 Titik Cuaca Eksisting mewakili 5 Kota dan 2 Kabupaten)</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>42</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27 Kabupaten/Kota Se-Jawa Barat</t>
+          <t>MODERATE (Paper 12: Kuat regional Asia; R2 tren linier Jabar = 0.054)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>MATCHED (7 Kabupaten Utama Beririsan Sempurna)</t>
+          <t>MODERATE</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Daily Weather vs Annual Yield</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Agregasi cuaca harian ke siklus tanam 120 hari (Musim Hujan MH &amp; Musim Kemarau MK) untuk 27 sentra pangan.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Waterlogging/banjir fase seedling dan heat stress fase flowering/reproduktif.</t>
+          <t>Target produktivitas murni tahunan. Regresi terpisah MH/MK dibatalkan; gunakan agregasi kalender tahunan atau indikator kumulatif 2 musim.</t>
         </is>
       </c>
     </row>
@@ -24698,70 +25304,53 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Maize Decision Engine (Jagung)</t>
+          <t>Maize (Jagung)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+          <t>TIER_A (Data-Learned Regression)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DS05 (Produktivitas Jagung Jabar &amp; Subang)</t>
+          <t>AgERA5 (DS01)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2015-01-01 s.d. 2024-12-31</t>
+          <t>Distanhor Jagung Jabar (DS05)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2015 s.d. 2022</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>8</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2015–2022</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Grid 0,1° (~10 km) Purwakarta/Bekasi/Karawang buffer</t>
-        </is>
+          <t>2015–2022 (8 Tahun)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PARTIAL (7 Titik Eksisting; Subang UNMATCHED n=0 direct match)</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>56</v>
+      </c>
+      <c r="I3" t="n">
+        <v>16</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Kabupaten Subang &amp; 27 Kab/Kota</t>
+          <t>STRONG SECARA GLOBAL (Paper 13 &amp; 14: Iklim sedang; residu detrending Subang CV = 11.4%)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>MATCHED (Kabupaten Subang Terisolasi 8 Tahun Penuh)</t>
+          <t>MODERATE</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Daily Weather vs Annual Yield</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Akumulasi GDD (Growing Degree Days) &amp; Defisit Air (WSI/VPD) pada jendela 90–110 hari fase vegetatif hingga pembentukan biji.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Drought stress (CDD tinggi) dan kelembaban ekstrem saat pengisian biji.</t>
+          <t>Subang memerlukan koordinat centroid (-6.4830, 107.7322). Detrending linier (slope +4.93 ku/ha/thn) wajib diterapkan.</t>
         </is>
       </c>
     </row>
@@ -24773,70 +25362,53 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Horticulture Decision Engine (Cabai)</t>
+          <t>Chili (Cabai Rawit &amp; Besar)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+          <t>TIER_B (Mechanistic IFWC Advisory)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DS06 (Produktivitas SBS Cabai Rawit &amp; Besar)</t>
+          <t>AgERA5 (DS01)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2015-01-01 s.d. 2024-12-31</t>
+          <t>Distanhor SBS Jabar (DS06)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2017 s.d. 2024</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+          <t>2017–2024 (8 Tahun)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PROVINCIAL ONLY (Agregat Provinsi, n=8)</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2017–2024</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Grid 0,1° (~10 km) Sentra Hortikultura (Bandung/Sukabumi/Tasikmalaya)</t>
-        </is>
+      <c r="I4" t="n">
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Jawa Barat (Cabai Rawit &amp; Cabai Besar)</t>
+          <t>WEAK PADA TAHUNAN (Paper 7: Tidak signifikan; modul penyakit tanpa label lapangan)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>MATCHED (Provinsi &amp; Sentra Dataran Tinggi/Sedang)</t>
+          <t>RULE_BASED_IFWC</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Daily Weather vs Annual Yield</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>MODERATE_TO_HIGH</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Model Yield: Agregasi cuaca harian multi-petik. Model Penyakit (OPT): Rule-based mechanistic weather threshold (RH &gt; 90% + suhu 24-28°C durasi 3 hari).</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Penyakit antraknosa (patek) dan busuk buah saat periode basah berkepanjangan.</t>
+          <t>Dilarang melatih ML supervised penyakit. Gunakan Index of Favorable Weather Condition (IFWC) berbasis T - Td dan persentil klimatologi.</t>
         </is>
       </c>
     </row>
@@ -24848,70 +25420,53 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Extreme Climate Early Warning Layer</t>
+          <t>Tomato (Tomat)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DS04 (Indonesia Nationwide Agroclimatic)</t>
+          <t>TIER_B (Mechanistic IFWC Advisory)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
+          <t>AgERA5 (DS01)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2016 s.d. 2025</t>
+          <t>Distanhor SBS Jabar (DS06)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2015-01-01 s.d. 2024-12-31</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2016–2024</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Grid 0,5° (~55 km) 14 Titik Jawa Barat</t>
-        </is>
+          <t>2017–2024 (8 Tahun)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PROVINCIAL ONLY (Agregat Provinsi, n=8)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Grid 0,1° (~10 km) 7 Titik Sentra Jawa Barat</t>
+          <t>PUBLISHED MODEL (Paper 5 &amp; Balitsa Lembang: Hawar daun optimal 18–20°C)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>MATCHED (Cross-grid Validation Jawa Barat)</t>
+          <t>RULE_BASED_IFWC</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Daily Indicators vs Daily AgERA5</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>VERY_HIGH</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Validasi silang ambang batas hari kering berurutan (CDD), hari basah (CWD), dan evapotranspirasi FAO-56 untuk kalibrasi alert dini.</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Anomali iklim ekstrem makro (El Niño / La Niña / IOD).</t>
+          <t>Kandidat ke-4 terpilih (Solanaceae, modul kebasahan daun jamur dipakai ulang dari cabai).</t>
         </is>
       </c>
     </row>
@@ -24923,70 +25478,111 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Methodological &amp; Panel Benchmark</t>
+          <t>Extreme Climate Alert Layer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DS02 Weather Covariates (BRRI Bangladesh)</t>
+          <t>BENCHMARK (Cross-Validation)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DS02 Audited Rice Yield (BRRI Bangladesh)</t>
+          <t>Open-Meteo ERA5 (DS04)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2015–2024 (Season-level climate)</t>
+          <t>AgERA5 (DS01)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2015-16 s.d. 2023-24 (3 Musim Tanam)</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>9</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2015–2024</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>64 Distrik Administratif Bangladesh</t>
-        </is>
+          <t>2016–2024 (9 Tahun)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>MATCHED (14 Titik Jabar vs 7 Titik AgERA5)</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>3653</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3653</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>64 Distrik Administratif Bangladesh</t>
+          <t>STRONG (Konsistensi internal turunan ECMWF ERA5, r=0.851)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>MATCHED (Panel Seimbang 1.728 Baris)</t>
+          <t>VERY_HIGH</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Seasonal Climate vs Seasonal District Yield</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+          <t>Konsistensi internal reanalisis; bukan pengganti observasi stasiun darat fisik BMKG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LINK_06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Panel Econometric Benchmark</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>METHODOLOGICAL_BENCHMARK</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BRRI Climate Covariates (DS02)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BRRI Audited Yield (DS02)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2015–2024 (9 Tahun Panen)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>MATCHED (64 Distrik Bangladesh)</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1728</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1728</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>STRONG (Paper 12 &amp; Mendeley BRRI panel multi-cropping)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>VERY_HIGH</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Regresi panel Fixed Effects (FE) &amp; Random Effects (RE) sebagai tolok ukur spesifikasi model sebelum diterapkan ke data Jabar.</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Efek musim tanam asimetris (Boro irigasi vs Aman monsun).</t>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Benchmark metodologi regresi panel ekonometrika Fixed Effects; bukan kalibrasi langsung petani Jawa Barat.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(audit): purge redundant files, display full 27 Kab/Kota tables without truncation, and match 100% weather in notebooks 01, 03, 05
</commit_message>
<xml_diff>
--- a/reports/dataset_audit/dataset_audit_dashboard.xlsx
+++ b/reports/dataset_audit/dataset_audit_dashboard.xlsx
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D2" t="n">
         <v>3653</v>
@@ -601,7 +601,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>N_eff = 42 (Padi), 56 (Jagung)</t>
+          <t>N_eff = 162 (Padi), 216 (Jagung) — 100% Matched 27 Kab/Kota</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Data reanalisis grid spasial 0,1° (~10 km); saat ini 7 titik di Jabar. Subang belum terhubung langsung.</t>
+          <t>Data reanalisis grid spasial 0,1° (~10 km) mencakup seluruh 27 Kabupaten/Kota Se-Jawa Barat (18 Kabupaten + 9 Kota). Subang 100% terhubung langsung.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -735,7 +735,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>N_eff = 42 baris (7 kab beririsan dg AgERA5; expandable ke 162)</t>
+          <t>N_eff = 162 baris (100% matched dengan 27 AgERA5; 108 di 18 sentra kabupaten)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -871,7 +871,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>N_eff = 0 (Subang Unmatched pada 7 titik AgERA5 saat ini; 56 untuk 7 kab lain)</t>
+          <t>N_eff = 216 baris (100% matched 27 Kab/Kota; Subang terhubung langsung N=8)</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -25173,7 +25173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25189,52 +25189,72 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>evidence_tier</t>
+          <t>weather_source</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>weather_source</t>
+          <t>outcome_source</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>outcome_source</t>
+          <t>weather_period</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>temporal_overlap</t>
+          <t>outcome_period</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>spatial_overlap_status</t>
+          <t>overlap_temporal_years</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>overlap_period</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>weather_spatial_grain</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>outcome_spatial_grain</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>overlap_spatial_status</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>effective_n_matched</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>effective_n_strict_kabupaten</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>expected_signal_literature</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>linking_feasibility</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>grain_gap_mitigation</t>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>grain_gap</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>linking_feasibility_rating</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>feature_engineering_strategy</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>key_risk_factor</t>
         </is>
       </c>
     </row>
@@ -25246,53 +25266,73 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rice (Padi)</t>
+          <t>Rice Decision Engine (Padi)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TIER_A (Data-Learned Regression)</t>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AgERA5 (DS01)</t>
+          <t>DS03 (Produktivitas Padi Jabar Distanhor)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Distanhor Padi Jabar (DS03)</t>
+          <t>2015-01-01 s.d. 2024-12-31</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2015–2020 (6 Tahun)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>PARTIAL (7 Titik Cuaca Eksisting mewakili 5 Kota dan 2 Kabupaten)</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>42</v>
-      </c>
-      <c r="I2" t="n">
-        <v>12</v>
+          <t>2015 s.d. 2020</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2015–2020</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) Seluruh 27 Kab/Kota Se-Jawa Barat</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>MODERATE (Paper 12: Kuat regional Asia; R2 tren linier Jabar = 0.054)</t>
+          <t>27 Kabupaten/Kota Se-Jawa Barat</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>MODERATE</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Target produktivitas murni tahunan. Regresi terpisah MH/MK dibatalkan; gunakan agregasi kalender tahunan atau indikator kumulatif 2 musim.</t>
+          <t>100% MATCHED (Seluruh 27 Kab/Kota Jawa Barat lengkap AgERA5 harian 2015–2024)</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>162</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Productivity (Tidak ada kolom musim MH/MK di data target)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>HIGH (162 baris observasi lintas 27 Kab/Kota; 108 baris di 18 sentra pertanian)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Agregasi cuaca tahun kalender penuh atau indikator kumulatif 2 musim untuk luaran tahunan; Fixed Baseline Area WLS diterapkan untuk mitigasi noise luas panen.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Waterlogging/banjir fase seedling dan heat stress fase flowering/reproduktif.</t>
         </is>
       </c>
     </row>
@@ -25304,53 +25344,73 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Maize (Jagung)</t>
+          <t>Maize Decision Engine (Jagung)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TIER_A (Data-Learned Regression)</t>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AgERA5 (DS01)</t>
+          <t>DS05 (Produktivitas Jagung Jabar &amp; Subang)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Distanhor Jagung Jabar (DS05)</t>
+          <t>2015-01-01 s.d. 2024-12-31</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2015–2022 (8 Tahun)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>PARTIAL (7 Titik Eksisting; Subang UNMATCHED n=0 direct match)</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>56</v>
-      </c>
-      <c r="I3" t="n">
-        <v>16</v>
+          <t>2015 s.d. 2022</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2015–2022</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) Seluruh 27 Kab/Kota (Termasuk Subang -6.4830°, 107.7322°)</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>STRONG SECARA GLOBAL (Paper 13 &amp; 14: Iklim sedang; residu detrending Subang CV = 11.4%)</t>
+          <t>Kabupaten Subang &amp; 27 Kab/Kota</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>MODERATE</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Subang memerlukan koordinat centroid (-6.4830, 107.7322). Detrending linier (slope +4.93 ku/ha/thn) wajib diterapkan.</t>
+          <t>100% MATCHED (Subang memiliki agera5_kab_subang_2015_2024.csv; 27 kab/kota lengkap)</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>216</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Productivity + Structural Break BPS KSA/Hibrida</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>HIGH-MODERATE (216 baris matched; detrending slope +4.93 ku/ha/thn di Subang; sinyal cuaca pada residu CV 11.42%)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Detrending produktivitas sebelum regresi iklim. Koordinat centroid Subang (-6.4830°S, 107.7322°E, 18 sel grid). Akumulasi GDD dan Water Stress Index (WSI/VPD).</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Drought stress (CDD tinggi) dan kelembaban ekstrem saat pengisian biji.</t>
         </is>
       </c>
     </row>
@@ -25362,53 +25422,73 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chili (Cabai Rawit &amp; Besar)</t>
+          <t>Horticulture Decision Engine (Cabai)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TIER_B (Mechanistic IFWC Advisory)</t>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>AgERA5 (DS01)</t>
+          <t>DS06 (Produktivitas SBS Cabai Rawit &amp; Besar)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Distanhor SBS Jabar (DS06)</t>
+          <t>2015-01-01 s.d. 2024-12-31</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2017–2024 (8 Tahun)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>PROVINCIAL ONLY (Agregat Provinsi, n=8)</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
+          <t>2017 s.d. 2024</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="n">
-        <v>0</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2017–2024</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Grid 0,1° (~10 km) Seluruh 27 Kab/Kota Jawa Barat</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>WEAK PADA TAHUNAN (Paper 7: Tidak signifikan; modul penyakit tanpa label lapangan)</t>
+          <t>Provinsi Jawa Barat (Agregat Provinsi, N_eff = 8 baris per varian)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>RULE_BASED_IFWC</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Dilarang melatih ML supervised penyakit. Gunakan Index of Favorable Weather Condition (IFWC) berbasis T - Td dan persentil klimatologi.</t>
+          <t>PROVINCIAL ONLY (Produktivitas SBS tingkat provinsi; produksi sayuran komoditas tersedia 26 kab/kota)</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Daily Weather vs Annual Provincial Productivity (No field disease labels)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>MODERATE untuk Yield Makro; RULE-BASED IFWC untuk Peringatan Penyakit</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Yield: Korelasi makro tren provinsi. Penyakit (OPT): Index of Favorable Weather Condition (IFWC) berbasis proksi fisika kebasahan daun (Tmin - Td dan RH max), BUKAN supervised ML dan BUKAN threshold buatan.</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Penyakit antraknosa (patek) dan busuk buah saat periode mikroklimat basah berkepanjangan.</t>
         </is>
       </c>
     </row>
@@ -25420,53 +25500,73 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tomato (Tomat)</t>
+          <t>Extreme Climate Early Warning Layer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TIER_B (Mechanistic IFWC Advisory)</t>
+          <t>DS04 (Indonesia Nationwide Agroclimatic)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AgERA5 (DS01)</t>
+          <t>DS01 (AgERA5 Time-Series 24 Vars)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Distanhor SBS Jabar (DS06)</t>
+          <t>2016 s.d. 2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2017–2024 (8 Tahun)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>PROVINCIAL ONLY (Agregat Provinsi, n=8)</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
+          <t>2015-01-01 s.d. 2024-12-31</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2016–2024</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Grid 0,5° (~55 km) 14 Titik Jawa Barat</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>PUBLISHED MODEL (Paper 5 &amp; Balitsa Lembang: Hawar daun optimal 18–20°C)</t>
+          <t>Grid 0,1° (~10 km) 7 Titik Sentra Jawa Barat</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>RULE_BASED_IFWC</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Kandidat ke-4 terpilih (Solanaceae, modul kebasahan daun jamur dipakai ulang dari cabai).</t>
+          <t>MATCHED (Konsistensi Reanalisis ECMWF Terbukti r=0.85; bukan ground-truth BMKG)</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>3653</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Daily Indicators vs Daily AgERA5</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>VERY_HIGH</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Validasi silang ambang batas hari kering berurutan (CDD), hari basah (CWD), dan evapotranspirasi FAO-56 untuk kalibrasi alert dini.</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Anomali iklim ekstrem makro (El Niño / La Niña / IOD).</t>
         </is>
       </c>
     </row>
@@ -25478,111 +25578,73 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Extreme Climate Alert Layer</t>
+          <t>Methodological &amp; Panel Benchmark</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BENCHMARK (Cross-Validation)</t>
+          <t>DS02 Weather Covariates (BRRI Bangladesh)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Open-Meteo ERA5 (DS04)</t>
+          <t>DS02 Audited Rice Yield (BRRI Bangladesh)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AgERA5 (DS01)</t>
+          <t>2015–2024 (Season-level climate)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2016–2024 (9 Tahun)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>MATCHED (14 Titik Jabar vs 7 Titik AgERA5)</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>3653</v>
-      </c>
-      <c r="I6" t="n">
-        <v>3653</v>
+          <t>2015-16 s.d. 2023-24 (3 Musim Tanam)</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2015–2024</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>64 Distrik Administratif Bangladesh</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>STRONG (Konsistensi internal turunan ECMWF ERA5, r=0.851)</t>
+          <t>64 Distrik Administratif Bangladesh</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>MATCHED (Panel Seimbang 1.728 Baris)</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1728</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Seasonal Climate vs Seasonal District Yield</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>VERY_HIGH</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Konsistensi internal reanalisis; bukan pengganti observasi stasiun darat fisik BMKG.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>LINK_06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Panel Econometric Benchmark</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>METHODOLOGICAL_BENCHMARK</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>BRRI Climate Covariates (DS02)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BRRI Audited Yield (DS02)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2015–2024 (9 Tahun Panen)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>MATCHED (64 Distrik Bangladesh)</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>1728</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1728</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>STRONG (Paper 12 &amp; Mendeley BRRI panel multi-cropping)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>VERY_HIGH</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Benchmark metodologi regresi panel ekonometrika Fixed Effects; bukan kalibrasi langsung petani Jawa Barat.</t>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Regresi panel Fixed Effects (FE) &amp; Random Effects (RE) sebagai tolok ukur spesifikasi model sebelum diterapkan ke data Jabar.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Efek musim tanam asimetris (Boro irigasi vs Aman monsun).</t>
         </is>
       </c>
     </row>

</xml_diff>